<commit_message>
Use reserved example domains in demo data; fix e-mail transliteration in project 05
</commit_message>
<xml_diff>
--- a/01-data-cleaning/output/clients_clean.xlsx
+++ b/01-data-cleaning/output/clients_clean.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -45,7 +48,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -53,13 +56,19 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -448,7 +457,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="31" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -501,7 +510,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>anna.nowak@gmail.com</t>
+          <t>anna.nowak@poczta.example</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -536,7 +545,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>jan.kowalski@firma.pl</t>
+          <t>jan.kowalski@firma.example</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -571,7 +580,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>piotr.wisniewski@wp.pl</t>
+          <t>piotr.wisniewski@mail.example</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -606,7 +615,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>k.wojcik@onet.pl</t>
+          <t>k.wojcik@skrzynka.example</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -641,7 +650,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>tomasz.kaminski@firma.com</t>
+          <t>tomasz.kaminski@firma.example</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -676,7 +685,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>magda.l@firma.pl</t>
+          <t>magda.l@firma.example</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -705,7 +714,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>b.szymanska@interia.pl</t>
+          <t>b.szymanska@list.example</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -740,7 +749,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>krzysztof@firma.pl</t>
+          <t>krzysztof@firma.example</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -775,7 +784,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ewa.dabrowska@firma.pl</t>
+          <t>ewa.dabrowska@firma.example</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -806,7 +815,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>michal.wozniak@firma.pl</t>
+          <t>michal.wozniak@firma.example</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -839,7 +848,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ola.mazur@gmail.com</t>
+          <t>ola.mazur@poczta.example</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -870,7 +879,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>robert.k@firma.pl</t>
+          <t>robert.k@firma.example</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -901,7 +910,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>g.jankowski@firma.pl</t>
+          <t>g.jankowski@firma.example</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -932,7 +941,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>monika.k@firma.pl</t>
+          <t>monika.k@firma.example</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">

</xml_diff>